<commit_message>
feat(bulk): refine SB collection compatibility
</commit_message>
<xml_diff>
--- a/bulk/src/assets/AmazonAdvertisingBulksheetSellerTemplate.xlsx
+++ b/bulk/src/assets/AmazonAdvertisingBulksheetSellerTemplate.xlsx
@@ -6,97 +6,99 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sponsored Brands Campaigns" r:id="rId3" sheetId="1"/>
-    <sheet name="SB Multi Ad Group Campaigns" r:id="rId4" sheetId="2"/>
+    <sheet name="Sponsored Display Campaigns" r:id="rId3" sheetId="1"/>
+    <sheet name="Portfolios" r:id="rId4" sheetId="2"/>
     <sheet name="RAS Campaigns" r:id="rId5" sheetId="3"/>
-    <sheet name="Sponsored Display Campaigns" r:id="rId6" sheetId="4"/>
-    <sheet name="Portfolios" r:id="rId7" sheetId="5"/>
-    <sheet name="Sponsored Products Campaigns" r:id="rId8" sheetId="6"/>
+    <sheet name="Sponsored Products Campaigns" r:id="rId6" sheetId="4"/>
+    <sheet name="Sponsored Brands Campaigns" r:id="rId7" sheetId="5"/>
+    <sheet name="SB Multi Ad Group Campaigns" r:id="rId8" sheetId="6"/>
     <sheet name="Config" r:id="rId9" sheetId="7" state="veryHidden"/>
   </sheets>
   <definedNames>
     <definedName name="SponsoredProductsProductNames">Config!$B$1:$B$1</definedName>
     <definedName name="SponsoredProductsEntityNames">Config!$B$2:$J$2</definedName>
     <definedName name="SponsoredProductsOperationNames">Config!$B$3:$D$3</definedName>
-    <definedName name="SponsoredProductsCreateCampaignNegativeKeywordMatchTypes">Config!$B$4:$C$4</definedName>
-    <definedName name="SponsoredProductsCreateKeywordMatchTypes">Config!$B$5:$D$5</definedName>
-    <definedName name="SponsoredProductsCreateNegativeKeywordMatchTypes">Config!$B$6:$C$6</definedName>
-    <definedName name="SponsoredProductsCreateCampaignTargetingTypes">Config!$B$7:$C$7</definedName>
-    <definedName name="SponsoredProductsCreateCampaignStates">Config!$B$8:$C$8</definedName>
-    <definedName name="SponsoredProductsUpdateCampaignStates">Config!$B$9:$D$9</definedName>
-    <definedName name="SponsoredProductsCreateCampaignNegativeKeywordStates">Config!$B$10:$B$10</definedName>
-    <definedName name="SponsoredProductsUpdateCampaignNegativeKeywordStates">Config!$B$11:$B$11</definedName>
-    <definedName name="SponsoredProductsCreateAdGroupStates">Config!$B$12:$C$12</definedName>
-    <definedName name="SponsoredProductsUpdateAdGroupStates">Config!$B$13:$D$13</definedName>
-    <definedName name="SponsoredProductsUpdateProductAdStates">Config!$B$14:$D$14</definedName>
-    <definedName name="SponsoredProductsCreateProductTargetingStates">Config!$B$15:$C$15</definedName>
-    <definedName name="SponsoredProductsUpdateProductTargetingStates">Config!$B$16:$D$16</definedName>
-    <definedName name="SponsoredProductsCreateNegativeProductTargetingStates">Config!$B$17:$C$17</definedName>
-    <definedName name="SponsoredProductsUpdateNegativeProductTargetingStates">Config!$B$18:$D$18</definedName>
-    <definedName name="SponsoredProductsCreateKeywordStates">Config!$B$19:$C$19</definedName>
-    <definedName name="SponsoredProductsUpdateKeywordStates">Config!$B$20:$D$20</definedName>
-    <definedName name="SponsoredProductsCreateNegativeKeywordStates">Config!$B$21:$C$21</definedName>
-    <definedName name="SponsoredProductsUpdateNegativeKeywordStates">Config!$B$22:$D$22</definedName>
-    <definedName name="SponsoredProductsCreateProductAdStates">Config!$B$23:$C$23</definedName>
-    <definedName name="SponsoredProductsCreateBiddingAdjustmentPlacements">Config!$B$24:$E$24</definedName>
-    <definedName name="SponsoredProductsUpdateBiddingAdjustmentPlacements">Config!$B$25:$E$25</definedName>
-    <definedName name="SponsoredProductsCreateCampaignStrategys">Config!$B$26:$D$26</definedName>
-    <definedName name="SponsoredProductsUpdateCampaignStrategys">Config!$B$27:$D$27</definedName>
-    <definedName name="SponsoredProductsCreateCampaignSiteRestrictions">Config!$B$28:$C$28</definedName>
-    <definedName name="SponsoredProductsCreateCampaignRequiredHeaders">Config!$B$29:$H$29</definedName>
-    <definedName name="SponsoredProductsUpdateCampaignRequiredHeaders">Config!$B$30:$G$30</definedName>
-    <definedName name="SponsoredProductsArchiveCampaignRequiredHeaders">Config!$B$31:$B$31</definedName>
-    <definedName name="SponsoredProductsCreateBiddingAdjustmentRequiredHeaders">Config!$B$32:$C$32</definedName>
-    <definedName name="SponsoredProductsUpdateBiddingAdjustmentRequiredHeaders">Config!$B$33:$C$33</definedName>
-    <definedName name="SponsoredProductsArchiveBiddingAdjustmentRequiredHeaders">Config!$B$34:$B$34</definedName>
-    <definedName name="SponsoredProductsCreateCampaignNegativeKeywordRequiredHeaders">Config!$B$35:$E$35</definedName>
-    <definedName name="SponsoredProductsUpdateCampaignNegativeKeywordRequiredHeaders">Config!$B$36:$C$36</definedName>
-    <definedName name="SponsoredProductsArchiveCampaignNegativeKeywordRequiredHeaders">Config!$B$37:$B$37</definedName>
-    <definedName name="SponsoredProductsCreateAdGroupRequiredHeaders">Config!$B$38:$F$38</definedName>
-    <definedName name="SponsoredProductsUpdateAdGroupRequiredHeaders">Config!$B$39:$E$39</definedName>
-    <definedName name="SponsoredProductsArchiveAdGroupRequiredHeaders">Config!$B$40:$B$40</definedName>
-    <definedName name="SponsoredProductsUpdateProductAdRequiredHeaders">Config!$B$41:$C$41</definedName>
-    <definedName name="SponsoredProductsArchiveProductAdRequiredHeaders">Config!$B$42:$B$42</definedName>
-    <definedName name="SponsoredProductsCreateProductTargetingRequiredHeaders">Config!$B$43:$E$43</definedName>
-    <definedName name="SponsoredProductsUpdateProductTargetingRequiredHeaders">Config!$B$44:$C$44</definedName>
-    <definedName name="SponsoredProductsArchiveProductTargetingRequiredHeaders">Config!$B$45:$B$45</definedName>
-    <definedName name="SponsoredProductsCreateNegativeProductTargetingRequiredHeaders">Config!$B$46:$E$46</definedName>
-    <definedName name="SponsoredProductsUpdateNegativeProductTargetingRequiredHeaders">Config!$B$47:$C$47</definedName>
-    <definedName name="SponsoredProductsArchiveNegativeProductTargetingRequiredHeaders">Config!$B$48:$B$48</definedName>
-    <definedName name="SponsoredProductsCreateKeywordRequiredHeaders">Config!$B$49:$F$49</definedName>
-    <definedName name="SponsoredProductsUpdateKeywordRequiredHeaders">Config!$B$50:$C$50</definedName>
-    <definedName name="SponsoredProductsArchiveKeywordRequiredHeaders">Config!$B$51:$B$51</definedName>
-    <definedName name="SponsoredProductsCreateNegativeKeywordRequiredHeaders">Config!$B$52:$F$52</definedName>
-    <definedName name="SponsoredProductsUpdateNegativeKeywordRequiredHeaders">Config!$B$53:$C$53</definedName>
-    <definedName name="SponsoredProductsArchiveNegativeKeywordRequiredHeaders">Config!$B$54:$B$54</definedName>
-    <definedName name="SponsoredProductsCreateProductAdRequiredHeaders">Config!$B$55:$E$55</definedName>
-    <definedName name="SponsoredProductsCreateCampaignOptionalHeaders">Config!$B$56:$D$56</definedName>
-    <definedName name="SponsoredProductsUpdateCampaignOptionalHeaders">Config!$B$57:$C$57</definedName>
-    <definedName name="SponsoredProductsArchiveCampaignOptionalHeaders">Config!$B$58:$A$58</definedName>
-    <definedName name="SponsoredProductsCreateBiddingAdjustmentOptionalHeaders">Config!$B$59:$B$59</definedName>
-    <definedName name="SponsoredProductsUpdateBiddingAdjustmentOptionalHeaders">Config!$B$60:$B$60</definedName>
-    <definedName name="SponsoredProductsArchiveBiddingAdjustmentOptionalHeaders">Config!$B$61:$A$61</definedName>
-    <definedName name="SponsoredProductsCreateCampaignNegativeKeywordOptionalHeaders">Config!$B$62:$A$62</definedName>
-    <definedName name="SponsoredProductsUpdateCampaignNegativeKeywordOptionalHeaders">Config!$B$63:$A$63</definedName>
-    <definedName name="SponsoredProductsArchiveCampaignNegativeKeywordOptionalHeaders">Config!$B$64:$A$64</definedName>
-    <definedName name="SponsoredProductsCreateAdGroupOptionalHeaders">Config!$B$65:$A$65</definedName>
-    <definedName name="SponsoredProductsUpdateAdGroupOptionalHeaders">Config!$B$66:$A$66</definedName>
-    <definedName name="SponsoredProductsArchiveAdGroupOptionalHeaders">Config!$B$67:$A$67</definedName>
-    <definedName name="SponsoredProductsUpdateProductAdOptionalHeaders">Config!$B$68:$A$68</definedName>
-    <definedName name="SponsoredProductsArchiveProductAdOptionalHeaders">Config!$B$69:$A$69</definedName>
-    <definedName name="SponsoredProductsCreateProductTargetingOptionalHeaders">Config!$B$70:$B$70</definedName>
-    <definedName name="SponsoredProductsUpdateProductTargetingOptionalHeaders">Config!$B$71:$B$71</definedName>
-    <definedName name="SponsoredProductsArchiveProductTargetingOptionalHeaders">Config!$B$72:$A$72</definedName>
-    <definedName name="SponsoredProductsCreateNegativeProductTargetingOptionalHeaders">Config!$B$73:$A$73</definedName>
-    <definedName name="SponsoredProductsUpdateNegativeProductTargetingOptionalHeaders">Config!$B$74:$A$74</definedName>
-    <definedName name="SponsoredProductsArchiveNegativeProductTargetingOptionalHeaders">Config!$B$75:$A$75</definedName>
-    <definedName name="SponsoredProductsCreateKeywordOptionalHeaders">Config!$B$76:$B$76</definedName>
-    <definedName name="SponsoredProductsUpdateKeywordOptionalHeaders">Config!$B$77:$B$77</definedName>
-    <definedName name="SponsoredProductsArchiveKeywordOptionalHeaders">Config!$B$78:$A$78</definedName>
-    <definedName name="SponsoredProductsCreateNegativeKeywordOptionalHeaders">Config!$B$79:$A$79</definedName>
-    <definedName name="SponsoredProductsUpdateNegativeKeywordOptionalHeaders">Config!$B$80:$A$80</definedName>
-    <definedName name="SponsoredProductsArchiveNegativeKeywordOptionalHeaders">Config!$B$81:$A$81</definedName>
-    <definedName name="SponsoredProductsCreateProductAdOptionalHeaders">Config!$B$82:$A$82</definedName>
+    <definedName name="SponsoredProductsCreateCampaignOffAmazonBudgetControlStrategys">Config!$B$4:$C$4</definedName>
+    <definedName name="SponsoredProductsUpdateCampaignOffAmazonBudgetControlStrategys">Config!$B$5:$C$5</definedName>
+    <definedName name="SponsoredProductsCreateCampaignNegativeKeywordMatchTypes">Config!$B$6:$C$6</definedName>
+    <definedName name="SponsoredProductsCreateKeywordMatchTypes">Config!$B$7:$D$7</definedName>
+    <definedName name="SponsoredProductsCreateNegativeKeywordMatchTypes">Config!$B$8:$C$8</definedName>
+    <definedName name="SponsoredProductsCreateCampaignTargetingTypes">Config!$B$9:$C$9</definedName>
+    <definedName name="SponsoredProductsCreateCampaignStates">Config!$B$10:$C$10</definedName>
+    <definedName name="SponsoredProductsUpdateCampaignStates">Config!$B$11:$D$11</definedName>
+    <definedName name="SponsoredProductsCreateCampaignNegativeKeywordStates">Config!$B$12:$B$12</definedName>
+    <definedName name="SponsoredProductsUpdateCampaignNegativeKeywordStates">Config!$B$13:$B$13</definedName>
+    <definedName name="SponsoredProductsCreateAdGroupStates">Config!$B$14:$C$14</definedName>
+    <definedName name="SponsoredProductsUpdateAdGroupStates">Config!$B$15:$D$15</definedName>
+    <definedName name="SponsoredProductsUpdateProductAdStates">Config!$B$16:$D$16</definedName>
+    <definedName name="SponsoredProductsCreateProductTargetingStates">Config!$B$17:$C$17</definedName>
+    <definedName name="SponsoredProductsUpdateProductTargetingStates">Config!$B$18:$D$18</definedName>
+    <definedName name="SponsoredProductsCreateNegativeProductTargetingStates">Config!$B$19:$C$19</definedName>
+    <definedName name="SponsoredProductsUpdateNegativeProductTargetingStates">Config!$B$20:$D$20</definedName>
+    <definedName name="SponsoredProductsCreateKeywordStates">Config!$B$21:$C$21</definedName>
+    <definedName name="SponsoredProductsUpdateKeywordStates">Config!$B$22:$D$22</definedName>
+    <definedName name="SponsoredProductsCreateNegativeKeywordStates">Config!$B$23:$C$23</definedName>
+    <definedName name="SponsoredProductsUpdateNegativeKeywordStates">Config!$B$24:$D$24</definedName>
+    <definedName name="SponsoredProductsCreateProductAdStates">Config!$B$25:$C$25</definedName>
+    <definedName name="SponsoredProductsCreateBiddingAdjustmentPlacements">Config!$B$26:$E$26</definedName>
+    <definedName name="SponsoredProductsUpdateBiddingAdjustmentPlacements">Config!$B$27:$E$27</definedName>
+    <definedName name="SponsoredProductsCreateCampaignStrategys">Config!$B$28:$D$28</definedName>
+    <definedName name="SponsoredProductsUpdateCampaignStrategys">Config!$B$29:$D$29</definedName>
+    <definedName name="SponsoredProductsCreateCampaignSiteRestrictions">Config!$B$30:$C$30</definedName>
+    <definedName name="SponsoredProductsCreateCampaignRequiredHeaders">Config!$B$31:$H$31</definedName>
+    <definedName name="SponsoredProductsUpdateCampaignRequiredHeaders">Config!$B$32:$G$32</definedName>
+    <definedName name="SponsoredProductsArchiveCampaignRequiredHeaders">Config!$B$33:$B$33</definedName>
+    <definedName name="SponsoredProductsCreateBiddingAdjustmentRequiredHeaders">Config!$B$34:$C$34</definedName>
+    <definedName name="SponsoredProductsUpdateBiddingAdjustmentRequiredHeaders">Config!$B$35:$C$35</definedName>
+    <definedName name="SponsoredProductsArchiveBiddingAdjustmentRequiredHeaders">Config!$B$36:$B$36</definedName>
+    <definedName name="SponsoredProductsCreateCampaignNegativeKeywordRequiredHeaders">Config!$B$37:$E$37</definedName>
+    <definedName name="SponsoredProductsUpdateCampaignNegativeKeywordRequiredHeaders">Config!$B$38:$C$38</definedName>
+    <definedName name="SponsoredProductsArchiveCampaignNegativeKeywordRequiredHeaders">Config!$B$39:$B$39</definedName>
+    <definedName name="SponsoredProductsCreateAdGroupRequiredHeaders">Config!$B$40:$F$40</definedName>
+    <definedName name="SponsoredProductsUpdateAdGroupRequiredHeaders">Config!$B$41:$E$41</definedName>
+    <definedName name="SponsoredProductsArchiveAdGroupRequiredHeaders">Config!$B$42:$B$42</definedName>
+    <definedName name="SponsoredProductsUpdateProductAdRequiredHeaders">Config!$B$43:$C$43</definedName>
+    <definedName name="SponsoredProductsArchiveProductAdRequiredHeaders">Config!$B$44:$B$44</definedName>
+    <definedName name="SponsoredProductsCreateProductTargetingRequiredHeaders">Config!$B$45:$E$45</definedName>
+    <definedName name="SponsoredProductsUpdateProductTargetingRequiredHeaders">Config!$B$46:$C$46</definedName>
+    <definedName name="SponsoredProductsArchiveProductTargetingRequiredHeaders">Config!$B$47:$B$47</definedName>
+    <definedName name="SponsoredProductsCreateNegativeProductTargetingRequiredHeaders">Config!$B$48:$E$48</definedName>
+    <definedName name="SponsoredProductsUpdateNegativeProductTargetingRequiredHeaders">Config!$B$49:$C$49</definedName>
+    <definedName name="SponsoredProductsArchiveNegativeProductTargetingRequiredHeaders">Config!$B$50:$B$50</definedName>
+    <definedName name="SponsoredProductsCreateKeywordRequiredHeaders">Config!$B$51:$F$51</definedName>
+    <definedName name="SponsoredProductsUpdateKeywordRequiredHeaders">Config!$B$52:$C$52</definedName>
+    <definedName name="SponsoredProductsArchiveKeywordRequiredHeaders">Config!$B$53:$B$53</definedName>
+    <definedName name="SponsoredProductsCreateNegativeKeywordRequiredHeaders">Config!$B$54:$F$54</definedName>
+    <definedName name="SponsoredProductsUpdateNegativeKeywordRequiredHeaders">Config!$B$55:$C$55</definedName>
+    <definedName name="SponsoredProductsArchiveNegativeKeywordRequiredHeaders">Config!$B$56:$B$56</definedName>
+    <definedName name="SponsoredProductsCreateProductAdRequiredHeaders">Config!$B$57:$E$57</definedName>
+    <definedName name="SponsoredProductsCreateCampaignOptionalHeaders">Config!$B$58:$E$58</definedName>
+    <definedName name="SponsoredProductsUpdateCampaignOptionalHeaders">Config!$B$59:$D$59</definedName>
+    <definedName name="SponsoredProductsArchiveCampaignOptionalHeaders">Config!$B$60:$A$60</definedName>
+    <definedName name="SponsoredProductsCreateBiddingAdjustmentOptionalHeaders">Config!$B$61:$B$61</definedName>
+    <definedName name="SponsoredProductsUpdateBiddingAdjustmentOptionalHeaders">Config!$B$62:$B$62</definedName>
+    <definedName name="SponsoredProductsArchiveBiddingAdjustmentOptionalHeaders">Config!$B$63:$A$63</definedName>
+    <definedName name="SponsoredProductsCreateCampaignNegativeKeywordOptionalHeaders">Config!$B$64:$A$64</definedName>
+    <definedName name="SponsoredProductsUpdateCampaignNegativeKeywordOptionalHeaders">Config!$B$65:$A$65</definedName>
+    <definedName name="SponsoredProductsArchiveCampaignNegativeKeywordOptionalHeaders">Config!$B$66:$A$66</definedName>
+    <definedName name="SponsoredProductsCreateAdGroupOptionalHeaders">Config!$B$67:$A$67</definedName>
+    <definedName name="SponsoredProductsUpdateAdGroupOptionalHeaders">Config!$B$68:$A$68</definedName>
+    <definedName name="SponsoredProductsArchiveAdGroupOptionalHeaders">Config!$B$69:$A$69</definedName>
+    <definedName name="SponsoredProductsUpdateProductAdOptionalHeaders">Config!$B$70:$A$70</definedName>
+    <definedName name="SponsoredProductsArchiveProductAdOptionalHeaders">Config!$B$71:$A$71</definedName>
+    <definedName name="SponsoredProductsCreateProductTargetingOptionalHeaders">Config!$B$72:$B$72</definedName>
+    <definedName name="SponsoredProductsUpdateProductTargetingOptionalHeaders">Config!$B$73:$B$73</definedName>
+    <definedName name="SponsoredProductsArchiveProductTargetingOptionalHeaders">Config!$B$74:$A$74</definedName>
+    <definedName name="SponsoredProductsCreateNegativeProductTargetingOptionalHeaders">Config!$B$75:$A$75</definedName>
+    <definedName name="SponsoredProductsUpdateNegativeProductTargetingOptionalHeaders">Config!$B$76:$A$76</definedName>
+    <definedName name="SponsoredProductsArchiveNegativeProductTargetingOptionalHeaders">Config!$B$77:$A$77</definedName>
+    <definedName name="SponsoredProductsCreateKeywordOptionalHeaders">Config!$B$78:$B$78</definedName>
+    <definedName name="SponsoredProductsUpdateKeywordOptionalHeaders">Config!$B$79:$B$79</definedName>
+    <definedName name="SponsoredProductsArchiveKeywordOptionalHeaders">Config!$B$80:$A$80</definedName>
+    <definedName name="SponsoredProductsCreateNegativeKeywordOptionalHeaders">Config!$B$81:$A$81</definedName>
+    <definedName name="SponsoredProductsUpdateNegativeKeywordOptionalHeaders">Config!$B$82:$A$82</definedName>
+    <definedName name="SponsoredProductsArchiveNegativeKeywordOptionalHeaders">Config!$B$83:$A$83</definedName>
+    <definedName name="SponsoredProductsCreateProductAdOptionalHeaders">Config!$B$84:$A$84</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -189,7 +191,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:V1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -215,32 +217,32 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Draft Campaign ID</t>
+          <t>Portfolio ID</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Portfolio ID</t>
+          <t>Ad Group ID</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Ad Group ID</t>
+          <t>Ad ID</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Keyword ID</t>
+          <t>Targeting ID</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Product Targeting ID</t>
+          <t>Campaign Name</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Campaign Name</t>
+          <t>Ad Group Name</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
@@ -260,97 +262,47 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>Tactic</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>Budget Type</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Ad Group Default Bid</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
         <is>
           <t>Bid Optimization</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Bid Multiplier</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Bid</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Keyword Text</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Match Type</t>
-        </is>
-      </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>Product Targeting Expression</t>
+          <t>Cost Type</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>Ad Format</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Landing Page URL</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Landing Page ASINs</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Brand Entity ID</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Brand Name</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Brand Logo Asset ID</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Custom Image Asset ID</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>Creative Headline</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>Creative ASINs</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>Video Media IDs</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>Creative Type</t>
+          <t>Targeting Expression</t>
         </is>
       </c>
     </row>
@@ -361,7 +313,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AR1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -382,207 +334,37 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Campaign ID</t>
+          <t>Portfolio ID</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Portfolio ID</t>
+          <t>Portfolio Name</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Ad Group ID</t>
+          <t>Budget Amount</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Ad ID</t>
+          <t>Budget Currency Code</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Keyword ID</t>
+          <t>Budget Policy</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Product Targeting ID</t>
+          <t>Budget Start Date</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Campaign Name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Ad Group Name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Ad Name</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>End Date</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Brand Entity ID</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Budget Type</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Budget</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Bid Optimization</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Product Location</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Bid</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Placement</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Percentage</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Audience ID</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Shopper Cohort Percentage</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Shopper Cohort Type</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Keyword Text</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Match Type</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>Native Language Keyword</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>Native Language Locale</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>Product Targeting Expression</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>Landing Page URL</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>Landing Page ASINs</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>Landing Page Type</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>Brand Name</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>Consent To Translate</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>Brand Logo Asset ID</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>Brand Logo Crop</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>Custom Images</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>Creative Headline</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>Creative ASINs</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
-        <is>
-          <t>Video Asset IDs</t>
-        </is>
-      </c>
-      <c r="AQ1" t="inlineStr">
-        <is>
-          <t>Subpages</t>
-        </is>
-      </c>
-      <c r="AR1" t="inlineStr">
-        <is>
-          <t>Sites</t>
+          <t>Budget End Date</t>
         </is>
       </c>
     </row>
@@ -750,7 +532,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -776,14 +558,14 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Ad Group ID</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Portfolio ID</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Ad Group ID</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
           <t>Ad ID</t>
@@ -791,47 +573,47 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Targeting ID</t>
+          <t>Keyword ID</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Product Targeting ID</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Ad Group Name</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Targeting Type</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Tactic</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Budget Type</t>
-        </is>
-      </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Daily Budget</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
@@ -851,28 +633,219 @@
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>Bid Optimization</t>
+          <t>Keyword Text</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>Cost Type</t>
+          <t>Native Language Keyword</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>Targeting Expression</t>
+          <t>Native Language Locale</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Match Type</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Bidding Strategy</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Placement</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Percentage</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Product Targeting Expression</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Audience ID</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Shopper Cohort Percentage</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>Shopper Cohort Type</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Off-Amazon ad serving</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="D2:AA1048576">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>IF($C2="",FALSE,COUNTIF(INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "RequiredHeaders")," ","")),D$1)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:AF1048576">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>IF($C2="",FALSE,COUNTIF(INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "OptionalHeaders")," ","")),F$1)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="43">
+    <dataValidation type="list" sqref="A2:A1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Product" error="Please choose one of the dropdown options." showErrorMessage="true">
+      <formula1>IF(A$1="Product", INDIRECT("SponsoredProductsProductNames"), "")</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="B2:B1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Entity" error="Please choose one of the dropdown options." showErrorMessage="true">
+      <formula1>IF(B$1="Entity", INDIRECT("SponsoredProductsEntityNames"), "")</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="C2:C1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Operation" error="Please choose one of the dropdown options." showErrorMessage="true">
+      <formula1>IF(C$1="Operation", INDIRECT("SponsoredProductsOperationNames"), "")</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="AF2:AF1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Off-Amazon ad serving" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="Off-Amazon ad serving" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
+      <formula1>IF(AF$1="Off-Amazon ad serving", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "OffAmazonBudgetControlStrategys"), " ", "")), "")</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="W2:W1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Match Type" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="Match Type" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
+      <formula1>IF(W$1="Match Type", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "MatchTypes"), " ", "")), "")</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="N2:N1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Targeting Type" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="Targeting Type" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
+      <formula1>IF(N$1="Targeting Type", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "TargetingTypes"), " ", "")), "")</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="O2:O1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid State" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="State" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
+      <formula1>IF(O$1="State", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "States"), " ", "")), "")</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="Y2:Y1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Placement" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="Placement" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
+      <formula1>IF(Y$1="Placement", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "Placements"), " ", "")), "")</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="X2:X1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Bidding Strategy" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="Bidding Strategy" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
+      <formula1>IF(X$1="Bidding Strategy", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "Strategys"), " ", "")), "")</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="AE2:AE1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Sites" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="Sites" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
+      <formula1>IF(AE$1="Sites", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "SiteRestrictions"), " ", "")), "")</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="R2:R1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Ad Group Default Bid" error="Ad Group Default Bid must be between 0.02 and 1000 and can have at most 2 decimal places. " showErrorMessage="true" promptTitle="Ad Group Default Bid" prompt="Ad Group Default Bid must be between 0.02 and 1000 and can have at most 2 decimal places. " showInputMessage="true">
+      <formula1>OR(R$1&lt;&gt;"Ad Group Default Bid", AND(AND($R2 &gt;= 0.02, $R2 &lt;= 1000),INT($R2*100)=$R2*100))</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="S2:S1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Bid" error="Bid must be between 0.02 and 1000 and can have at most 2 decimal places. " showErrorMessage="true" promptTitle="Bid" prompt="Bid must be between 0.02 and 1000 and can have at most 2 decimal places. " showInputMessage="true">
+      <formula1>OR(S$1&lt;&gt;"Bid", AND(AND($S2 &gt;= 0.02, $S2 &lt;= 1000),INT($S2*100)=$S2*100))</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="P2:P1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Daily Budget" error="Daily Budget must be between 1 and 1000000 and can have at most 2 decimal places. " showErrorMessage="true" promptTitle="Daily Budget" prompt="Daily Budget must be between 1 and 1000000 and can have at most 2 decimal places. " showInputMessage="true">
+      <formula1>OR(P$1&lt;&gt;"Daily Budget", AND(AND($P2 &gt;= 1, $P2 &lt;= 1000000),INT($P2*100)=$P2*100))</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="J2:J1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Campaign Name" error="Campaign Name can have up to 128 characters. " showErrorMessage="true" promptTitle="Campaign Name" prompt="Campaign Name can have up to 128 characters. " showInputMessage="true">
+      <formula1>OR(J$1&lt;&gt;"Campaign Name", AND(LEN($J2) &lt;= 128))</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="K2:K1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Ad Group Name" error="Ad Group Name can have up to 255 characters. " showErrorMessage="true" promptTitle="Ad Group Name" prompt="Ad Group Name can have up to 255 characters. " showInputMessage="true">
+      <formula1>OR(K$1&lt;&gt;"Ad Group Name", AND(LEN($K2) &lt;= 255))</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="L2:L1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Start Date" error="Start Date must be formatted as YYYYMMDD and must be today or in the future. " showErrorMessage="true" promptTitle="Start Date" prompt="Start Date must be formatted as YYYYMMDD and must be today or in the future. " showInputMessage="true">
+      <formula1>OR(L$1&lt;&gt;"Start Date", AND(LEN($L2)=8,DATEVALUE(REPLACE(REPLACE($L2,7,0,"/"),5,0,"/"))&gt;=TODAY()))</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="M2:M1048576" allowBlank="false" errorStyle="information" errorTitle="Invalid End Date" error="End Date must be formatted as YYYYMMDD and must occur after the start date. " showErrorMessage="true" promptTitle="End Date" prompt="End Date must be formatted as YYYYMMDD and must occur after the start date. " showInputMessage="true">
+      <formula1>OR(M$1&lt;&gt;"End Date", AND(OR(LEN($M2)=0,AND(LEN($M2)=8,IFERROR(DATEVALUE(REPLACE(REPLACE($M2,7,0,"/"),5,0,"/")),-1)&gt;=IF(LEN($L2)&lt;&gt;8,0,IFERROR(DATEVALUE(REPLACE(REPLACE($L2,7,0,"/"),5,0,"/")),0))))))</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="Z2:Z1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Percentage" error="Percentage can have at most 2 decimal places. " showErrorMessage="true" promptTitle="Percentage" prompt="Percentage can have at most 2 decimal places. " showInputMessage="true">
+      <formula1>OR(Z$1&lt;&gt;"Percentage", AND(INT($Z2*100)=$Z2*100))</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="AC2:AC1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Shopper Cohort Percentage" error="Shopper Cohort Percentage can have at most 2 decimal places. " showErrorMessage="true" promptTitle="Shopper Cohort Percentage" prompt="Shopper Cohort Percentage can have at most 2 decimal places. " showInputMessage="true">
+      <formula1>OR(AC$1&lt;&gt;"Shopper Cohort Percentage", AND(INT($AC2*100)=$AC2*100))</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="A1" allowBlank="true" errorStyle="stop" promptTitle="Product" prompt="Enter the sponsored ads campaign type here." showInputMessage="true">
+      <formula1>A$1="Product"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="B1" allowBlank="true" errorStyle="stop" promptTitle="Entity" prompt="Select the entity that you want to manage." showInputMessage="true">
+      <formula1>B$1="Entity"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="C1" allowBlank="true" errorStyle="stop" promptTitle="Operation" prompt="Enter an action you want to perform in this row. If this cell is blank, the row will be ignored. After you select an Entity and Operation, some fields in the row will highlight to indicate which need values. Dark blue = required, light blue = optional." showInputMessage="true">
+      <formula1>C$1="Operation"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="D1" allowBlank="true" errorStyle="stop" promptTitle="Campaign Id" prompt="To create a Campaign, choose a temporary ID starting with a letter. Enter the exact same ID to create child entities for the Campaign. This will become a system-generated ID when the Campaign is created. To update the Campaign, use the system-generated ID" showInputMessage="true">
+      <formula1>D$1="Campaign Id"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="E1" allowBlank="true" errorStyle="stop" promptTitle="Ad Group Id" prompt="To create an Ad Group, choose a temporary ID starting with a letter. Enter the exact same ID to create child entities in the Ad Group. This will become a system-generated ID when the Ad Group is created. To update the Ad Group, use the system-generated ID" showInputMessage="true">
+      <formula1>E$1="Ad Group Id"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="F1" allowBlank="true" errorStyle="stop" promptTitle="Portfolio Id" prompt="You can add a campaign to an existing portfolio by adding the Portfolio ID here. The Portfolio must be created in the Portfolio sheet or Ads Console beforehand." showInputMessage="true">
+      <formula1>F$1="Portfolio Id"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="G1" allowBlank="true" errorStyle="stop" promptTitle="Ad Id" prompt="Ensure Ad ID is entered when updating Product Ad. An ID is not needed in this field if you are creating a new Product Ad." showInputMessage="true">
+      <formula1>G$1="Ad Id"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="H1" allowBlank="true" errorStyle="stop" promptTitle="Keyword Id" prompt="Ensure Keyword ID is entered when updating Keyword, Negative Keyword, or Campaign Negative Keyword. An ID is not needed in this field if you are creating a new Keyword." showInputMessage="true">
+      <formula1>H$1="Keyword Id"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="I1" allowBlank="true" errorStyle="stop" promptTitle="Product Targeting Id" prompt="Ensure Product Targeting ID is entered when updating Product Targeting or Negative Product Targeting. An ID is not needed in this field if you are creating new Targeting." showInputMessage="true">
+      <formula1>I$1="Product Targeting Id"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="J1" allowBlank="true" errorStyle="stop" promptTitle="Campaign Name" prompt="Create or update Campaign Name here. Non-English language is acceptable. Name must not exceed 128 characters." showInputMessage="true">
+      <formula1>J$1="Campaign Name"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="K1" allowBlank="true" errorStyle="stop" promptTitle="Ad Group Name" prompt="Create or update Ad Group Name here. Non-English language is acceptable. Name must not exceed 255 characters." showInputMessage="true">
+      <formula1>K$1="Ad Group Name"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="O1" allowBlank="true" errorStyle="stop" promptTitle="State" prompt="Enter a status to create or update entities. You do not need to enter or change a status if you are archiving." showInputMessage="true">
+      <formula1>O$1="State"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="L1" allowBlank="true" errorStyle="stop" promptTitle="Start Date" prompt="Start date must occur in the future. Use format YYYYMMDD (April 15, 2023 would be 20230415)." showInputMessage="true">
+      <formula1>L$1="Start Date"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="M1" allowBlank="true" errorStyle="stop" promptTitle="End Date" prompt="Use format YYYYMMDD (April 15, 2023 would be 20230415). If left blank, the campaign will run indefinitely." showInputMessage="true">
+      <formula1>M$1="End Date"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="Q1" allowBlank="true" errorStyle="stop" promptTitle="SKU" prompt="Enter the SKU code to create Product Ads with seller accounts." showInputMessage="true">
+      <formula1>Q$1="SKU"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="T1" allowBlank="true" errorStyle="stop" promptTitle="Keyword Text" prompt="Limited to 80 characters max per keyword. Avoid these symbols: slashes, carets, commas, double periods. Non-English language is acceptable." showInputMessage="true">
+      <formula1>T$1="Keyword Text"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="Z1" allowBlank="true" errorStyle="stop" promptTitle="Percentage" prompt="Enter percent amount to create or update bidding adjustment by placement. Percent symbol (%) isn’t needed (e.g., enter 10.25 if allocating 10.25%)." showInputMessage="true">
+      <formula1>Z$1="Percentage"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="Y1" allowBlank="true" errorStyle="stop" promptTitle="Placement" prompt="When creating a bidding adjustment, enter placementTop for top-of-search, or placementProductPage for product page placements." showInputMessage="true">
+      <formula1>Y$1="Placement"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="AB1" allowBlank="true" errorStyle="stop" promptTitle="Audience ID" prompt="To create a bidding adjustment by shopper cohort, enter the audience ID associated with an audience segment." showInputMessage="true">
+      <formula1>AB$1="Audience ID"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="AD1" allowBlank="true" errorStyle="stop" promptTitle="Shopper Cohort Type" prompt="Enter the type of shopper cohort type to create or update bidding adjustment by shopper cohort. Currently, the only supported type is AUDIENCE_SEGMENT." showInputMessage="true">
+      <formula1>AD$1="Shopper Cohort Type"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="AC1" allowBlank="true" errorStyle="stop" promptTitle="Shopper Cohort Percentage" prompt="Enter percent amount to create or update bidding adjustment by shopper cohort. Percent symbol (%) isn’t needed (e.g., enter 10.25 if allocating 10.25%)." showInputMessage="true">
+      <formula1>AC$1="Shopper Cohort Percentage"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="AA1" allowBlank="true" errorStyle="stop" promptTitle="Product Targeting Expression" prompt="Enter the code for the category, product, brand, and so on. Codes can be found in the Resolved Targeting Expression field in a downloaded bulksheet. Use the format asin=&quot;AXXXXXXXXX&quot;, category = &quot;XXX&quot;, brand=&quot;XXX&quot;." showInputMessage="true">
+      <formula1>AA$1="Product Targeting Expression"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="AE1" allowBlank="true" errorStyle="stop" promptTitle="Sites" prompt="Sites are where specific ad placements can appear. These can be websites or apps." showInputMessage="true">
+      <formula1>AE$1="Sites"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" sqref="AF1" allowBlank="true" errorStyle="stop" promptTitle="Off-Amazon ad serving" prompt="Off-Amazon ad serving_x000a_Increase reach: Increase your reach off Amazon. This setting may result in more impressions and opportunities for sales off Amazon_x000a_Limit off-Amazon spend: Reduce spend off Amazon for low-performing placements." showInputMessage="true">
+      <formula1>AF$1="Off-Amazon ad serving"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -893,37 +866,147 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Campaign ID</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Draft Campaign ID</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Portfolio ID</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Portfolio Name</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Budget Amount</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Budget Currency Code</t>
+          <t>Ad Group ID</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Budget Policy</t>
+          <t>Keyword ID</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Budget Start Date</t>
+          <t>Product Targeting ID</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Budget End Date</t>
+          <t>Campaign Name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Budget Type</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Bid Optimization</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Bid Multiplier</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Keyword Text</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Match Type</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Product Targeting Expression</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Ad Format</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Landing Page URL</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Landing Page ASINs</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Brand Entity ID</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Brand Name</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Brand Logo Asset ID</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Custom Image Asset ID</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Creative Headline</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>Creative ASINs</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>Video Media IDs</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Creative Type</t>
         </is>
       </c>
     </row>
@@ -934,7 +1017,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AT1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -960,14 +1043,14 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Portfolio ID</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Ad Group ID</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Portfolio ID</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
           <t>Ad ID</t>
@@ -995,19 +1078,19 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>Ad Name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Targeting Type</t>
-        </is>
-      </c>
       <c r="O1" t="inlineStr">
         <is>
           <t>State</t>
@@ -1015,228 +1098,168 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Daily Budget</t>
+          <t>Brand Entity ID</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Budget Type</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>Ad Group Default Bid</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
+          <t>Bid Optimization</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Product Location</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
           <t>Bid</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Placement</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Percentage</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Audience ID</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Shopper Cohort Percentage</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Shopper Cohort Type</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Keyword Text</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Match Type</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Native Language Keyword</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Native Language Locale</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Match Type</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Bidding Strategy</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Placement</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Percentage</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Product Targeting Expression</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Audience ID</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>Shopper Cohort Percentage</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>Shopper Cohort Type</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Landing Page URL</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Landing Page ASINs</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>Landing Page Type</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>Brand Name</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>Consent To Translate</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>Brand Logo Asset ID</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>Brand Logo Crop</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>Custom Images</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>Creative Headline</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>Creative ASINs</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>Video Asset IDs</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>Subpages</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>Product Exclusions</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>Ad Title</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
         <is>
           <t>Sites</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:AA1048576">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>IF($C2="",FALSE,COUNTIF(INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "RequiredHeaders")," ","")),D$1)&gt;0)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:AE1048576">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>IF($C2="",FALSE,COUNTIF(INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "OptionalHeaders")," ","")),F$1)&gt;0)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="41">
-    <dataValidation type="list" sqref="A2:A1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Product" error="Please choose one of the dropdown options." showErrorMessage="true">
-      <formula1>IF(A$1="Product", INDIRECT("SponsoredProductsProductNames"), "")</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="B2:B1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Entity" error="Please choose one of the dropdown options." showErrorMessage="true">
-      <formula1>IF(B$1="Entity", INDIRECT("SponsoredProductsEntityNames"), "")</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="C2:C1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Operation" error="Please choose one of the dropdown options." showErrorMessage="true">
-      <formula1>IF(C$1="Operation", INDIRECT("SponsoredProductsOperationNames"), "")</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="W2:W1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Match Type" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="Match Type" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
-      <formula1>IF(W$1="Match Type", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "MatchTypes"), " ", "")), "")</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="N2:N1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Targeting Type" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="Targeting Type" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
-      <formula1>IF(N$1="Targeting Type", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "TargetingTypes"), " ", "")), "")</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="O2:O1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid State" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="State" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
-      <formula1>IF(O$1="State", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "States"), " ", "")), "")</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="Y2:Y1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Placement" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="Placement" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
-      <formula1>IF(Y$1="Placement", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "Placements"), " ", "")), "")</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="X2:X1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Bidding Strategy" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="Bidding Strategy" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
-      <formula1>IF(X$1="Bidding Strategy", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "Strategys"), " ", "")), "")</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="AE2:AE1048576" allowBlank="true" errorStyle="information" showDropDown="false" errorTitle="Invalid Sites" error="Please choose one of the dropdown options." showErrorMessage="true" promptTitle="Sites" prompt="If dropdown options are not appearing, this means that the operation is blank or this cell is not editable. Using cut/paste can also break the dropdown rules._x000a_" showInputMessage="true">
-      <formula1>IF(AE$1="Sites", INDIRECT(SUBSTITUTE(CONCATENATE($A2, $C2, $B2, "SiteRestrictions"), " ", "")), "")</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="R2:R1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Ad Group Default Bid" error="Ad Group Default Bid must be between 0.02 and 1000 and can have at most 2 decimal places. " showErrorMessage="true" promptTitle="Ad Group Default Bid" prompt="Ad Group Default Bid must be between 0.02 and 1000 and can have at most 2 decimal places. " showInputMessage="true">
-      <formula1>OR(R$1&lt;&gt;"Ad Group Default Bid", AND(AND($R2 &gt;= 0.02, $R2 &lt;= 1000),INT($R2*100)=$R2*100))</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="S2:S1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Bid" error="Bid must be between 0.02 and 1000 and can have at most 2 decimal places. " showErrorMessage="true" promptTitle="Bid" prompt="Bid must be between 0.02 and 1000 and can have at most 2 decimal places. " showInputMessage="true">
-      <formula1>OR(S$1&lt;&gt;"Bid", AND(AND($S2 &gt;= 0.02, $S2 &lt;= 1000),INT($S2*100)=$S2*100))</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="P2:P1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Daily Budget" error="Daily Budget must be between 1 and 1000000 and can have at most 2 decimal places. " showErrorMessage="true" promptTitle="Daily Budget" prompt="Daily Budget must be between 1 and 1000000 and can have at most 2 decimal places. " showInputMessage="true">
-      <formula1>OR(P$1&lt;&gt;"Daily Budget", AND(AND($P2 &gt;= 1, $P2 &lt;= 1000000),INT($P2*100)=$P2*100))</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="J2:J1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Campaign Name" error="Campaign Name can have up to 128 characters. " showErrorMessage="true" promptTitle="Campaign Name" prompt="Campaign Name can have up to 128 characters. " showInputMessage="true">
-      <formula1>OR(J$1&lt;&gt;"Campaign Name", AND(LEN($J2) &lt;= 128))</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="K2:K1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Ad Group Name" error="Ad Group Name can have up to 255 characters. " showErrorMessage="true" promptTitle="Ad Group Name" prompt="Ad Group Name can have up to 255 characters. " showInputMessage="true">
-      <formula1>OR(K$1&lt;&gt;"Ad Group Name", AND(LEN($K2) &lt;= 255))</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="L2:L1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Start Date" error="Start Date must be formatted as YYYYMMDD and must be today or in the future. " showErrorMessage="true" promptTitle="Start Date" prompt="Start Date must be formatted as YYYYMMDD and must be today or in the future. " showInputMessage="true">
-      <formula1>OR(L$1&lt;&gt;"Start Date", AND(LEN($L2)=8,DATEVALUE(REPLACE(REPLACE($L2,7,0,"/"),5,0,"/"))&gt;=TODAY()))</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="M2:M1048576" allowBlank="false" errorStyle="information" errorTitle="Invalid End Date" error="End Date must be formatted as YYYYMMDD and must occur after the start date. " showErrorMessage="true" promptTitle="End Date" prompt="End Date must be formatted as YYYYMMDD and must occur after the start date. " showInputMessage="true">
-      <formula1>OR(M$1&lt;&gt;"End Date", AND(OR(LEN($M2)=0,AND(LEN($M2)=8,IFERROR(DATEVALUE(REPLACE(REPLACE($M2,7,0,"/"),5,0,"/")),-1)&gt;=IF(LEN($L2)&lt;&gt;8,0,IFERROR(DATEVALUE(REPLACE(REPLACE($L2,7,0,"/"),5,0,"/")),0))))))</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="Z2:Z1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Percentage" error="Percentage can have at most 2 decimal places. " showErrorMessage="true" promptTitle="Percentage" prompt="Percentage can have at most 2 decimal places. " showInputMessage="true">
-      <formula1>OR(Z$1&lt;&gt;"Percentage", AND(INT($Z2*100)=$Z2*100))</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="AC2:AC1048576" allowBlank="true" errorStyle="information" errorTitle="Invalid Shopper Cohort Percentage" error="Shopper Cohort Percentage can have at most 2 decimal places. " showErrorMessage="true" promptTitle="Shopper Cohort Percentage" prompt="Shopper Cohort Percentage can have at most 2 decimal places. " showInputMessage="true">
-      <formula1>OR(AC$1&lt;&gt;"Shopper Cohort Percentage", AND(INT($AC2*100)=$AC2*100))</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="A1" allowBlank="true" errorStyle="stop" promptTitle="Product" prompt="Enter the sponsored ads campaign type here." showInputMessage="true">
-      <formula1>A$1="Product"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="B1" allowBlank="true" errorStyle="stop" promptTitle="Entity" prompt="Select the entity that you want to manage." showInputMessage="true">
-      <formula1>B$1="Entity"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="C1" allowBlank="true" errorStyle="stop" promptTitle="Operation" prompt="Enter an action you want to perform in this row. If this cell is blank, the row will be ignored. After you select an Entity and Operation, some fields in the row will highlight to indicate which need values. Dark blue = required, light blue = optional." showInputMessage="true">
-      <formula1>C$1="Operation"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="D1" allowBlank="true" errorStyle="stop" promptTitle="Campaign Id" prompt="To create a Campaign, choose a temporary ID starting with a letter. Enter the exact same ID to create child entities for the Campaign. This will become a system-generated ID when the Campaign is created. To update the Campaign, use the system-generated ID" showInputMessage="true">
-      <formula1>D$1="Campaign Id"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="E1" allowBlank="true" errorStyle="stop" promptTitle="Ad Group Id" prompt="To create an Ad Group, choose a temporary ID starting with a letter. Enter the exact same ID to create child entities in the Ad Group. This will become a system-generated ID when the Ad Group is created. To update the Ad Group, use the system-generated ID" showInputMessage="true">
-      <formula1>E$1="Ad Group Id"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="F1" allowBlank="true" errorStyle="stop" promptTitle="Portfolio Id" prompt="You can add a campaign to an existing portfolio by adding the Portfolio ID here. The Portfolio must be created in the Portfolio sheet or Ads Console beforehand." showInputMessage="true">
-      <formula1>F$1="Portfolio Id"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="G1" allowBlank="true" errorStyle="stop" promptTitle="Ad Id" prompt="Ensure Ad ID is entered when updating Product Ad. An ID is not needed in this field if you are creating a new Product Ad." showInputMessage="true">
-      <formula1>G$1="Ad Id"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="H1" allowBlank="true" errorStyle="stop" promptTitle="Keyword Id" prompt="Ensure Keyword ID is entered when updating Keyword, Negative Keyword, or Campaign Negative Keyword. An ID is not needed in this field if you are creating a new Keyword." showInputMessage="true">
-      <formula1>H$1="Keyword Id"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="I1" allowBlank="true" errorStyle="stop" promptTitle="Product Targeting Id" prompt="Ensure Product Targeting ID is entered when updating Product Targeting or Negative Product Targeting. An ID is not needed in this field if you are creating new Targeting." showInputMessage="true">
-      <formula1>I$1="Product Targeting Id"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="J1" allowBlank="true" errorStyle="stop" promptTitle="Campaign Name" prompt="Create or update Campaign Name here. Non-English language is acceptable. Name must not exceed 128 characters." showInputMessage="true">
-      <formula1>J$1="Campaign Name"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="K1" allowBlank="true" errorStyle="stop" promptTitle="Ad Group Name" prompt="Create or update Ad Group Name here. Non-English language is acceptable. Name must not exceed 255 characters." showInputMessage="true">
-      <formula1>K$1="Ad Group Name"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="O1" allowBlank="true" errorStyle="stop" promptTitle="State" prompt="Enter a status to create or update entities. You do not need to enter or change a status if you are archiving." showInputMessage="true">
-      <formula1>O$1="State"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="L1" allowBlank="true" errorStyle="stop" promptTitle="Start Date" prompt="Start date must occur in the future. Use format YYYYMMDD (April 15, 2023 would be 20230415)." showInputMessage="true">
-      <formula1>L$1="Start Date"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="M1" allowBlank="true" errorStyle="stop" promptTitle="End Date" prompt="Use format YYYYMMDD (April 15, 2023 would be 20230415). If left blank, the campaign will run indefinitely." showInputMessage="true">
-      <formula1>M$1="End Date"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="Q1" allowBlank="true" errorStyle="stop" promptTitle="SKU" prompt="Enter the SKU code to create Product Ads with seller accounts." showInputMessage="true">
-      <formula1>Q$1="SKU"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="T1" allowBlank="true" errorStyle="stop" promptTitle="Keyword Text" prompt="Limited to 80 characters max per keyword. Avoid these symbols: slashes, carets, commas, double periods. Non-English language is acceptable." showInputMessage="true">
-      <formula1>T$1="Keyword Text"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="Z1" allowBlank="true" errorStyle="stop" promptTitle="Percentage" prompt="Enter percent amount to create or update bidding adjustment by placement. Percent symbol (%) isn’t needed (e.g., enter 10.25 if allocating 10.25%)." showInputMessage="true">
-      <formula1>Z$1="Percentage"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="Y1" allowBlank="true" errorStyle="stop" promptTitle="Placement" prompt="When creating a bidding adjustment, enter placementTop for top-of-search, or placementProductPage for product page placements." showInputMessage="true">
-      <formula1>Y$1="Placement"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="AB1" allowBlank="true" errorStyle="stop" promptTitle="Audience ID" prompt="To create a bidding adjustment by shopper cohort, enter the audience ID associated with an audience segment." showInputMessage="true">
-      <formula1>AB$1="Audience ID"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="AD1" allowBlank="true" errorStyle="stop" promptTitle="Shopper Cohort Type" prompt="Enter the type of shopper cohort type to create or update bidding adjustment by shopper cohort. Currently, the only supported type is AUDIENCE_SEGMENT." showInputMessage="true">
-      <formula1>AD$1="Shopper Cohort Type"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="AC1" allowBlank="true" errorStyle="stop" promptTitle="Shopper Cohort Percentage" prompt="Enter percent amount to create or update bidding adjustment by shopper cohort. Percent symbol (%) isn’t needed (e.g., enter 10.25 if allocating 10.25%)." showInputMessage="true">
-      <formula1>AC$1="Shopper Cohort Percentage"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="AA1" allowBlank="true" errorStyle="stop" promptTitle="Product Targeting Expression" prompt="Enter the code for the category, product, brand, and so on. Codes can be found in the Resolved Targeting Expression field in a downloaded bulksheet. Use the format asin=&quot;AXXXXXXXXX&quot;, category = &quot;XXX&quot;, brand=&quot;XXX&quot;." showInputMessage="true">
-      <formula1>AA$1="Product Targeting Expression"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" sqref="AE1" allowBlank="true" errorStyle="stop" promptTitle="Sites" prompt="Sites are where specific ad placements can appear. These can be websites or apps." showInputMessage="true">
-      <formula1>AE$1="Sites"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1328,46 +1351,41 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateCampaignNegativeKeywordMatchTypes</t>
+          <t>SponsoredProductsCreateCampaignOffAmazonBudgetControlStrategys</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>negativeExact</t>
+          <t>Increase reach</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>negativePhrase</t>
+          <t>Limit off-Amazon spend</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateKeywordMatchTypes</t>
+          <t>SponsoredProductsUpdateCampaignOffAmazonBudgetControlStrategys</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>Increase reach</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>phrase</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>broad</t>
+          <t>Limit off-Amazon spend</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateNegativeKeywordMatchTypes</t>
+          <t>SponsoredProductsCreateCampaignNegativeKeywordMatchTypes</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1384,78 +1402,93 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateCampaignTargetingTypes</t>
+          <t>SponsoredProductsCreateKeywordMatchTypes</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AUTO</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>phrase</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>broad</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateCampaignStates</t>
+          <t>SponsoredProductsCreateNegativeKeywordMatchTypes</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>negativeExact</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>paused</t>
+          <t>negativePhrase</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateCampaignStates</t>
+          <t>SponsoredProductsCreateCampaignTargetingTypes</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>AUTO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>paused</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>archived</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateCampaignNegativeKeywordStates</t>
+          <t>SponsoredProductsCreateCampaignStates</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
           <t>enabled</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>paused</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateCampaignNegativeKeywordStates</t>
+          <t>SponsoredProductsUpdateCampaignStates</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>archived</t>
         </is>
@@ -1464,37 +1497,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateAdGroupStates</t>
+          <t>SponsoredProductsCreateCampaignNegativeKeywordStates</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>enabled</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>paused</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateAdGroupStates</t>
+          <t>SponsoredProductsUpdateCampaignNegativeKeywordStates</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
-        <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>paused</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
         <is>
           <t>archived</t>
         </is>
@@ -1503,7 +1521,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateProductAdStates</t>
+          <t>SponsoredProductsCreateAdGroupStates</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1514,18 +1532,13 @@
       <c r="C14" t="inlineStr">
         <is>
           <t>paused</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>archived</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateProductTargetingStates</t>
+          <t>SponsoredProductsUpdateAdGroupStates</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1536,13 +1549,18 @@
       <c r="C15" t="inlineStr">
         <is>
           <t>paused</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>archived</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateProductTargetingStates</t>
+          <t>SponsoredProductsUpdateProductAdStates</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1564,7 +1582,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateNegativeProductTargetingStates</t>
+          <t>SponsoredProductsCreateProductTargetingStates</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1581,7 +1599,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateNegativeProductTargetingStates</t>
+          <t>SponsoredProductsUpdateProductTargetingStates</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1603,7 +1621,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateKeywordStates</t>
+          <t>SponsoredProductsCreateNegativeProductTargetingStates</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1620,7 +1638,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateKeywordStates</t>
+          <t>SponsoredProductsUpdateNegativeProductTargetingStates</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1642,7 +1660,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateNegativeKeywordStates</t>
+          <t>SponsoredProductsCreateKeywordStates</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1659,7 +1677,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateNegativeKeywordStates</t>
+          <t>SponsoredProductsUpdateKeywordStates</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1681,7 +1699,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateProductAdStates</t>
+          <t>SponsoredProductsCreateNegativeKeywordStates</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1698,213 +1716,203 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateBiddingAdjustmentPlacements</t>
+          <t>SponsoredProductsUpdateNegativeKeywordStates</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>placementTop</t>
+          <t>enabled</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>placementProductPage</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>placementRestOfSearch</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>placementAmazonBusiness</t>
+          <t>archived</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateBiddingAdjustmentPlacements</t>
+          <t>SponsoredProductsCreateProductAdStates</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>placementTop</t>
+          <t>enabled</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>placementProductPage</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>placementRestOfSearch</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>placementAmazonBusiness</t>
+          <t>paused</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateCampaignStrategys</t>
+          <t>SponsoredProductsCreateBiddingAdjustmentPlacements</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>placementTop</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dynamic bids - up and down</t>
+          <t>placementProductPage</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Fixed bid</t>
+          <t>placementRestOfSearch</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>placementAmazonBusiness</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateCampaignStrategys</t>
+          <t>SponsoredProductsUpdateBiddingAdjustmentPlacements</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Dynamic bids - down only</t>
+          <t>placementTop</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Dynamic bids - up and down</t>
+          <t>placementProductPage</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Fixed bid</t>
+          <t>placementRestOfSearch</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>placementAmazonBusiness</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateCampaignSiteRestrictions</t>
+          <t>SponsoredProductsCreateCampaignStrategys</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Amazon Business</t>
+          <t>Dynamic bids - down only</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Amazon Haul</t>
+          <t>Dynamic bids - up and down</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateCampaignRequiredHeaders</t>
+          <t>SponsoredProductsUpdateCampaignStrategys</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Campaign Id</t>
+          <t>Dynamic bids - down only</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Campaign Name</t>
+          <t>Dynamic bids - up and down</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Daily Budget</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Targeting Type</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Bidding Strategy</t>
+          <t>Fixed bid</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateCampaignRequiredHeaders</t>
+          <t>SponsoredProductsCreateCampaignSiteRestrictions</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Campaign Id</t>
+          <t>Amazon Business</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Campaign Name</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Daily Budget</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Bidding Strategy</t>
+          <t>Amazon Haul</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveCampaignRequiredHeaders</t>
+          <t>SponsoredProductsCreateCampaignRequiredHeaders</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
           <t>Campaign Id</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Campaign Name</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Daily Budget</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Targeting Type</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Bidding Strategy</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateBiddingAdjustmentRequiredHeaders</t>
+          <t>SponsoredProductsUpdateCampaignRequiredHeaders</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1914,43 +1922,63 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Placement</t>
+          <t>Campaign Name</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Daily Budget</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Bidding Strategy</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateBiddingAdjustmentRequiredHeaders</t>
+          <t>SponsoredProductsArchiveCampaignRequiredHeaders</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
           <t>Campaign Id</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Placement</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveBiddingAdjustmentRequiredHeaders</t>
+          <t>SponsoredProductsCreateBiddingAdjustmentRequiredHeaders</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
           <t>Campaign Id</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Placement</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateCampaignNegativeKeywordRequiredHeaders</t>
+          <t>SponsoredProductsUpdateBiddingAdjustmentRequiredHeaders</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1960,76 +1988,61 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Keyword Text</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Match Type</t>
+          <t>Placement</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateCampaignNegativeKeywordRequiredHeaders</t>
+          <t>SponsoredProductsArchiveBiddingAdjustmentRequiredHeaders</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Keyword Id</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>State</t>
+          <t>Campaign Id</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveCampaignNegativeKeywordRequiredHeaders</t>
+          <t>SponsoredProductsCreateCampaignNegativeKeywordRequiredHeaders</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Keyword Id</t>
+          <t>Campaign Id</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Keyword Text</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Match Type</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateAdGroupRequiredHeaders</t>
+          <t>SponsoredProductsUpdateCampaignNegativeKeywordRequiredHeaders</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Campaign Id</t>
+          <t>Keyword Id</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
-        <is>
-          <t>Ad Group Id</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Ad Group Name</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Ad Group Default Bid</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
         <is>
           <t>State</t>
         </is>
@@ -2038,54 +2051,69 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateAdGroupRequiredHeaders</t>
+          <t>SponsoredProductsArchiveCampaignNegativeKeywordRequiredHeaders</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Ad Group Id</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Ad Group Name</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Ad Group Default Bid</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>State</t>
+          <t>Keyword Id</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveAdGroupRequiredHeaders</t>
+          <t>SponsoredProductsCreateAdGroupRequiredHeaders</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>Campaign Id</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
           <t>Ad Group Id</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Ad Group Name</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Ad Group Default Bid</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>State</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateProductAdRequiredHeaders</t>
+          <t>SponsoredProductsUpdateAdGroupRequiredHeaders</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ad Id</t>
+          <t>Ad Group Id</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
+        <is>
+          <t>Ad Group Name</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Ad Group Default Bid</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>State</t>
         </is>
@@ -2094,271 +2122,261 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveProductAdRequiredHeaders</t>
+          <t>SponsoredProductsArchiveAdGroupRequiredHeaders</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ad Id</t>
+          <t>Ad Group Id</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateProductTargetingRequiredHeaders</t>
+          <t>SponsoredProductsUpdateProductAdRequiredHeaders</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Campaign Id</t>
+          <t>Ad Id</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Ad Group Id</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
           <t>State</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Product Targeting Expression</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateProductTargetingRequiredHeaders</t>
+          <t>SponsoredProductsArchiveProductAdRequiredHeaders</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Product Targeting Id</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>State</t>
+          <t>Ad Id</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveProductTargetingRequiredHeaders</t>
+          <t>SponsoredProductsCreateProductTargetingRequiredHeaders</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Product Targeting Id</t>
+          <t>Campaign Id</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Ad Group Id</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Product Targeting Expression</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateNegativeProductTargetingRequiredHeaders</t>
+          <t>SponsoredProductsUpdateProductTargetingRequiredHeaders</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Campaign Id</t>
+          <t>Product Targeting Id</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Ad Group Id</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
           <t>State</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Product Targeting Expression</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateNegativeProductTargetingRequiredHeaders</t>
+          <t>SponsoredProductsArchiveProductTargetingRequiredHeaders</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
           <t>Product Targeting Id</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>State</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveNegativeProductTargetingRequiredHeaders</t>
+          <t>SponsoredProductsCreateNegativeProductTargetingRequiredHeaders</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Product Targeting Id</t>
+          <t>Campaign Id</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Ad Group Id</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Product Targeting Expression</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateKeywordRequiredHeaders</t>
+          <t>SponsoredProductsUpdateNegativeProductTargetingRequiredHeaders</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Campaign Id</t>
+          <t>Product Targeting Id</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Ad Group Id</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
           <t>State</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Keyword Text</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Match Type</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateKeywordRequiredHeaders</t>
+          <t>SponsoredProductsArchiveNegativeProductTargetingRequiredHeaders</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Keyword Id</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>State</t>
+          <t>Product Targeting Id</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveKeywordRequiredHeaders</t>
+          <t>SponsoredProductsCreateKeywordRequiredHeaders</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Keyword Id</t>
+          <t>Campaign Id</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Ad Group Id</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Keyword Text</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Match Type</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateNegativeKeywordRequiredHeaders</t>
+          <t>SponsoredProductsUpdateKeywordRequiredHeaders</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Campaign Id</t>
+          <t>Keyword Id</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Ad Group Id</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
           <t>State</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Keyword Text</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Match Type</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateNegativeKeywordRequiredHeaders</t>
+          <t>SponsoredProductsArchiveKeywordRequiredHeaders</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
           <t>Keyword Id</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>State</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveNegativeKeywordRequiredHeaders</t>
+          <t>SponsoredProductsCreateNegativeKeywordRequiredHeaders</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Keyword Id</t>
+          <t>Campaign Id</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Ad Group Id</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Keyword Text</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Match Type</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateProductAdRequiredHeaders</t>
+          <t>SponsoredProductsUpdateNegativeKeywordRequiredHeaders</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Campaign Id</t>
+          <t>Keyword Id</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
-        <is>
-          <t>Ad Group Id</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
         <is>
           <t>State</t>
         </is>
@@ -2367,242 +2385,291 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateCampaignOptionalHeaders</t>
+          <t>SponsoredProductsArchiveNegativeKeywordRequiredHeaders</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Portfolio Id</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>End Date</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Sites</t>
+          <t>Keyword Id</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateCampaignOptionalHeaders</t>
+          <t>SponsoredProductsCreateProductAdRequiredHeaders</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Portfolio Id</t>
+          <t>Campaign Id</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>End Date</t>
+          <t>Ad Group Id</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>State</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveCampaignOptionalHeaders</t>
+          <t>SponsoredProductsCreateCampaignOptionalHeaders</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Portfolio Id</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Off-Amazon ad serving</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateBiddingAdjustmentOptionalHeaders</t>
+          <t>SponsoredProductsUpdateCampaignOptionalHeaders</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Percentage</t>
+          <t>Portfolio Id</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Off-Amazon ad serving</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateBiddingAdjustmentOptionalHeaders</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Percentage</t>
+          <t>SponsoredProductsArchiveCampaignOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveBiddingAdjustmentOptionalHeaders</t>
+          <t>SponsoredProductsCreateBiddingAdjustmentOptionalHeaders</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Percentage</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateCampaignNegativeKeywordOptionalHeaders</t>
+          <t>SponsoredProductsUpdateBiddingAdjustmentOptionalHeaders</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Percentage</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateCampaignNegativeKeywordOptionalHeaders</t>
+          <t>SponsoredProductsArchiveBiddingAdjustmentOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveCampaignNegativeKeywordOptionalHeaders</t>
+          <t>SponsoredProductsCreateCampaignNegativeKeywordOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateAdGroupOptionalHeaders</t>
+          <t>SponsoredProductsUpdateCampaignNegativeKeywordOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateAdGroupOptionalHeaders</t>
+          <t>SponsoredProductsArchiveCampaignNegativeKeywordOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveAdGroupOptionalHeaders</t>
+          <t>SponsoredProductsCreateAdGroupOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateProductAdOptionalHeaders</t>
+          <t>SponsoredProductsUpdateAdGroupOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveProductAdOptionalHeaders</t>
+          <t>SponsoredProductsArchiveAdGroupOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateProductTargetingOptionalHeaders</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Bid</t>
+          <t>SponsoredProductsUpdateProductAdOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateProductTargetingOptionalHeaders</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Bid</t>
+          <t>SponsoredProductsArchiveProductAdOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveProductTargetingOptionalHeaders</t>
+          <t>SponsoredProductsCreateProductTargetingOptionalHeaders</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Bid</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateNegativeProductTargetingOptionalHeaders</t>
+          <t>SponsoredProductsUpdateProductTargetingOptionalHeaders</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Bid</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateNegativeProductTargetingOptionalHeaders</t>
+          <t>SponsoredProductsArchiveProductTargetingOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveNegativeProductTargetingOptionalHeaders</t>
+          <t>SponsoredProductsCreateNegativeProductTargetingOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateKeywordOptionalHeaders</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Bid</t>
+          <t>SponsoredProductsUpdateNegativeProductTargetingOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateKeywordOptionalHeaders</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Bid</t>
+          <t>SponsoredProductsArchiveNegativeProductTargetingOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveKeywordOptionalHeaders</t>
+          <t>SponsoredProductsCreateKeywordOptionalHeaders</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Bid</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SponsoredProductsCreateNegativeKeywordOptionalHeaders</t>
+          <t>SponsoredProductsUpdateKeywordOptionalHeaders</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Bid</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SponsoredProductsUpdateNegativeKeywordOptionalHeaders</t>
+          <t>SponsoredProductsArchiveKeywordOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SponsoredProductsArchiveNegativeKeywordOptionalHeaders</t>
+          <t>SponsoredProductsCreateNegativeKeywordOptionalHeaders</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
+        <is>
+          <t>SponsoredProductsUpdateNegativeKeywordOptionalHeaders</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>SponsoredProductsArchiveNegativeKeywordOptionalHeaders</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
         <is>
           <t>SponsoredProductsCreateProductAdOptionalHeaders</t>
         </is>

</xml_diff>